<commit_message>
menambahkan logger.js dan integrasi log di index.js
</commit_message>
<xml_diff>
--- a/MigrasiDanaAnggota.xlsx
+++ b/MigrasiDanaAnggota.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TOMOSTUFF\KoperasiGKPS_Railway\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C5B363-088D-4196-B7C4-FE6CF5063F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85DAEB51-0330-49CF-8206-6CE1DD31023C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{7A9B5D7B-9D1F-4191-8DEC-E5161677A5EB}"/>
   </bookViews>
@@ -25,16 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
-  <si>
-    <t>0613001</t>
-  </si>
-  <si>
-    <t>0613003</t>
-  </si>
-  <si>
-    <t>0613004</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>0613005</t>
   </si>
@@ -611,16 +602,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" t="s">
         <v>66</v>
-      </c>
-      <c r="B1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -631,10 +622,10 @@
         <v>100000</v>
       </c>
       <c r="C2">
-        <v>1970000</v>
+        <v>170000</v>
       </c>
       <c r="D2">
-        <v>1950000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -645,7 +636,7 @@
         <v>100000</v>
       </c>
       <c r="C3">
-        <v>1210000</v>
+        <v>1930000</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -659,7 +650,7 @@
         <v>100000</v>
       </c>
       <c r="C4">
-        <v>800000</v>
+        <v>490000</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -673,10 +664,10 @@
         <v>100000</v>
       </c>
       <c r="C5">
-        <v>170000</v>
+        <v>2030000</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -687,7 +678,7 @@
         <v>100000</v>
       </c>
       <c r="C6">
-        <v>1930000</v>
+        <v>820000</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -701,7 +692,7 @@
         <v>100000</v>
       </c>
       <c r="C7">
-        <v>490000</v>
+        <v>100000</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -715,10 +706,10 @@
         <v>100000</v>
       </c>
       <c r="C8">
-        <v>2030000</v>
+        <v>1970000</v>
       </c>
       <c r="D8">
-        <v>300000</v>
+        <v>1400000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -729,10 +720,10 @@
         <v>100000</v>
       </c>
       <c r="C9">
-        <v>820000</v>
+        <v>2170000</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -743,10 +734,10 @@
         <v>100000</v>
       </c>
       <c r="C10">
-        <v>100000</v>
+        <v>2170000</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -757,10 +748,10 @@
         <v>100000</v>
       </c>
       <c r="C11">
-        <v>1970000</v>
+        <v>2170000</v>
       </c>
       <c r="D11">
-        <v>1400000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -771,10 +762,10 @@
         <v>100000</v>
       </c>
       <c r="C12">
-        <v>2170000</v>
+        <v>1920000</v>
       </c>
       <c r="D12">
-        <v>1440000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -785,10 +776,10 @@
         <v>100000</v>
       </c>
       <c r="C13">
-        <v>2170000</v>
+        <v>1650000</v>
       </c>
       <c r="D13">
-        <v>1440000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -799,10 +790,10 @@
         <v>100000</v>
       </c>
       <c r="C14">
-        <v>2170000</v>
+        <v>1020000</v>
       </c>
       <c r="D14">
-        <v>500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -813,7 +804,7 @@
         <v>100000</v>
       </c>
       <c r="C15">
-        <v>1920000</v>
+        <v>600000</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -827,7 +818,7 @@
         <v>100000</v>
       </c>
       <c r="C16">
-        <v>1650000</v>
+        <v>1900000</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -841,7 +832,7 @@
         <v>100000</v>
       </c>
       <c r="C17">
-        <v>1020000</v>
+        <v>1410000</v>
       </c>
       <c r="D17">
         <v>0</v>
@@ -855,7 +846,7 @@
         <v>100000</v>
       </c>
       <c r="C18">
-        <v>600000</v>
+        <v>1390000</v>
       </c>
       <c r="D18">
         <v>0</v>
@@ -869,7 +860,7 @@
         <v>100000</v>
       </c>
       <c r="C19">
-        <v>1900000</v>
+        <v>2020000</v>
       </c>
       <c r="D19">
         <v>0</v>
@@ -883,7 +874,7 @@
         <v>100000</v>
       </c>
       <c r="C20">
-        <v>1410000</v>
+        <v>1160000</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -897,7 +888,7 @@
         <v>100000</v>
       </c>
       <c r="C21">
-        <v>1390000</v>
+        <v>1880000</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -911,7 +902,7 @@
         <v>100000</v>
       </c>
       <c r="C22">
-        <v>2020000</v>
+        <v>2230000</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -925,7 +916,7 @@
         <v>100000</v>
       </c>
       <c r="C23">
-        <v>1160000</v>
+        <v>1690000</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -939,7 +930,7 @@
         <v>100000</v>
       </c>
       <c r="C24">
-        <v>1880000</v>
+        <v>920000</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -953,7 +944,7 @@
         <v>100000</v>
       </c>
       <c r="C25">
-        <v>2230000</v>
+        <v>920000</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -967,7 +958,7 @@
         <v>100000</v>
       </c>
       <c r="C26">
-        <v>1690000</v>
+        <v>1910000</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -981,10 +972,10 @@
         <v>100000</v>
       </c>
       <c r="C27">
-        <v>920000</v>
+        <v>2150000</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -995,7 +986,7 @@
         <v>100000</v>
       </c>
       <c r="C28">
-        <v>920000</v>
+        <v>730000</v>
       </c>
       <c r="D28">
         <v>0</v>
@@ -1009,7 +1000,7 @@
         <v>100000</v>
       </c>
       <c r="C29">
-        <v>1910000</v>
+        <v>1900000</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -1023,10 +1014,10 @@
         <v>100000</v>
       </c>
       <c r="C30">
-        <v>2150000</v>
+        <v>910000</v>
       </c>
       <c r="D30">
-        <v>1440000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1037,7 +1028,7 @@
         <v>100000</v>
       </c>
       <c r="C31">
-        <v>730000</v>
+        <v>1560000</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1051,7 +1042,7 @@
         <v>100000</v>
       </c>
       <c r="C32">
-        <v>1900000</v>
+        <v>650000</v>
       </c>
       <c r="D32">
         <v>0</v>
@@ -1065,7 +1056,7 @@
         <v>100000</v>
       </c>
       <c r="C33">
-        <v>910000</v>
+        <v>1790000</v>
       </c>
       <c r="D33">
         <v>0</v>
@@ -1079,7 +1070,7 @@
         <v>100000</v>
       </c>
       <c r="C34">
-        <v>1560000</v>
+        <v>660000</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -1093,7 +1084,7 @@
         <v>100000</v>
       </c>
       <c r="C35">
-        <v>650000</v>
+        <v>250000</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1107,7 +1098,7 @@
         <v>100000</v>
       </c>
       <c r="C36">
-        <v>1790000</v>
+        <v>350000</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1121,7 +1112,7 @@
         <v>100000</v>
       </c>
       <c r="C37">
-        <v>660000</v>
+        <v>1700000</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -1135,7 +1126,7 @@
         <v>100000</v>
       </c>
       <c r="C38">
-        <v>250000</v>
+        <v>1425000</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -1149,7 +1140,7 @@
         <v>100000</v>
       </c>
       <c r="C39">
-        <v>350000</v>
+        <v>170000</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -1163,7 +1154,7 @@
         <v>100000</v>
       </c>
       <c r="C40">
-        <v>1700000</v>
+        <v>480000</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1177,7 +1168,7 @@
         <v>100000</v>
       </c>
       <c r="C41">
-        <v>1425000</v>
+        <v>1370000</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -1191,7 +1182,7 @@
         <v>100000</v>
       </c>
       <c r="C42">
-        <v>170000</v>
+        <v>1430000</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -1205,7 +1196,7 @@
         <v>100000</v>
       </c>
       <c r="C43">
-        <v>480000</v>
+        <v>550000</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -1219,7 +1210,7 @@
         <v>100000</v>
       </c>
       <c r="C44">
-        <v>1370000</v>
+        <v>1240000</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -1233,7 +1224,7 @@
         <v>100000</v>
       </c>
       <c r="C45">
-        <v>1430000</v>
+        <v>1120000</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -1247,7 +1238,7 @@
         <v>100000</v>
       </c>
       <c r="C46">
-        <v>550000</v>
+        <v>1100000</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -1261,7 +1252,7 @@
         <v>100000</v>
       </c>
       <c r="C47">
-        <v>1240000</v>
+        <v>970000</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -1275,10 +1266,10 @@
         <v>100000</v>
       </c>
       <c r="C48">
-        <v>1120000</v>
+        <v>900000</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -1289,10 +1280,10 @@
         <v>100000</v>
       </c>
       <c r="C49">
-        <v>1100000</v>
+        <v>880000</v>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1303,10 +1294,10 @@
         <v>100000</v>
       </c>
       <c r="C50">
-        <v>970000</v>
+        <v>950000</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1317,10 +1308,10 @@
         <v>100000</v>
       </c>
       <c r="C51">
-        <v>900000</v>
+        <v>950000</v>
       </c>
       <c r="D51">
-        <v>40000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1331,10 +1322,10 @@
         <v>100000</v>
       </c>
       <c r="C52">
-        <v>880000</v>
+        <v>740000</v>
       </c>
       <c r="D52">
-        <v>200000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1345,10 +1336,10 @@
         <v>100000</v>
       </c>
       <c r="C53">
-        <v>950000</v>
+        <v>890000</v>
       </c>
       <c r="D53">
-        <v>500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1359,10 +1350,10 @@
         <v>100000</v>
       </c>
       <c r="C54">
-        <v>950000</v>
+        <v>10000</v>
       </c>
       <c r="D54">
-        <v>500000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1373,7 +1364,7 @@
         <v>100000</v>
       </c>
       <c r="C55">
-        <v>740000</v>
+        <v>880000</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -1387,7 +1378,7 @@
         <v>100000</v>
       </c>
       <c r="C56">
-        <v>890000</v>
+        <v>650000</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -1401,7 +1392,7 @@
         <v>100000</v>
       </c>
       <c r="C57">
-        <v>10000</v>
+        <v>870000</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -1415,7 +1406,7 @@
         <v>100000</v>
       </c>
       <c r="C58">
-        <v>880000</v>
+        <v>710000</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -1429,7 +1420,7 @@
         <v>100000</v>
       </c>
       <c r="C59">
-        <v>650000</v>
+        <v>870000</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -1443,10 +1434,10 @@
         <v>100000</v>
       </c>
       <c r="C60">
-        <v>870000</v>
+        <v>860000</v>
       </c>
       <c r="D60">
-        <v>0</v>
+        <v>1950000</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1457,7 +1448,7 @@
         <v>100000</v>
       </c>
       <c r="C61">
-        <v>710000</v>
+        <v>520000</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -1471,7 +1462,7 @@
         <v>100000</v>
       </c>
       <c r="C62">
-        <v>870000</v>
+        <v>20000</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -1485,10 +1476,10 @@
         <v>100000</v>
       </c>
       <c r="C63">
-        <v>860000</v>
+        <v>60000</v>
       </c>
       <c r="D63">
-        <v>1950000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -1499,55 +1490,13 @@
         <v>100000</v>
       </c>
       <c r="C64">
-        <v>520000</v>
+        <v>400000</v>
       </c>
       <c r="D64">
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>63</v>
-      </c>
-      <c r="B65">
-        <v>100000</v>
-      </c>
-      <c r="C65">
-        <v>20000</v>
-      </c>
-      <c r="D65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>64</v>
-      </c>
-      <c r="B66">
-        <v>100000</v>
-      </c>
-      <c r="C66">
-        <v>60000</v>
-      </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>65</v>
-      </c>
-      <c r="B67">
-        <v>100000</v>
-      </c>
-      <c r="C67">
-        <v>400000</v>
-      </c>
-      <c r="D67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>

</xml_diff>

<commit_message>
feat: integrasi full audit log di semua endpoint utama
</commit_message>
<xml_diff>
--- a/MigrasiDanaAnggota.xlsx
+++ b/MigrasiDanaAnggota.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TOMOSTUFF\KoperasiGKPS_Railway\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85DAEB51-0330-49CF-8206-6CE1DD31023C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75599DCC-B923-4EB7-9CB6-93F162E180E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{7A9B5D7B-9D1F-4191-8DEC-E5161677A5EB}"/>
   </bookViews>
@@ -252,12 +252,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -273,9 +279,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -839,16 +846,16 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B18">
-        <v>100000</v>
-      </c>
-      <c r="C18">
+      <c r="B18" s="2">
+        <v>100000</v>
+      </c>
+      <c r="C18" s="2">
         <v>1390000</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>